<commit_message>
rename two metric limits to follow conventions
</commit_message>
<xml_diff>
--- a/python/pdstools/resources/MetricLimits.xlsx
+++ b/python/pdstools/resources/MetricLimits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kass1/Documents/Code/pdstools_v4/pega-datascientist-tools/python/pdstools/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanej/Code/pega-datascientist-tools/python/pdstools/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7D033C-1DA4-8543-B0E1-A332D4DD7A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD10626C-7A66-8949-AD0E-C63600C1C113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="880" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -221,12 +221,6 @@
     <t>ActiveActionCount</t>
   </si>
   <si>
-    <t>AverageGroupsPerIssue</t>
-  </si>
-  <si>
-    <t>AverageTreatmentsPerChannelPerAction</t>
-  </si>
-  <si>
     <t>InactiveActionCount</t>
   </si>
   <si>
@@ -264,6 +258,12 @@
   </si>
   <si>
     <t>ModelsWithoutResponsesPercentage</t>
+  </si>
+  <si>
+    <t>TreatmentsPerChannelPerActionAverage</t>
+  </si>
+  <si>
+    <t>GroupsPerIssueAverage</t>
   </si>
 </sst>
 </file>
@@ -827,7 +827,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C6" s="11">
         <v>0.75</v>
@@ -842,7 +842,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C7" s="11">
         <v>0.75</v>
@@ -911,7 +911,7 @@
         <v>19</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C12" s="1">
         <v>-4</v>
@@ -920,7 +920,7 @@
         <v>-2</v>
       </c>
       <c r="G12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H12" s="6"/>
     </row>
@@ -1079,7 +1079,7 @@
         <v>26</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C23" s="10">
         <v>0.5</v>
@@ -1111,7 +1111,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
@@ -1320,7 +1320,7 @@
         <v>58</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C40" s="3">
         <v>1</v>
@@ -1340,7 +1340,7 @@
         <v>58</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C41" s="3">
         <v>1</v>
@@ -1360,7 +1360,7 @@
         <v>58</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1368,7 +1368,7 @@
         <v>58</v>
       </c>
       <c r="B43" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C43" s="3">
         <v>1</v>
@@ -1385,7 +1385,7 @@
         <v>58</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C44" s="3">
         <v>1</v>
@@ -1405,7 +1405,7 @@
         <v>58</v>
       </c>
       <c r="B45" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C45" s="3">
         <v>2</v>
@@ -1428,7 +1428,7 @@
         <v>58</v>
       </c>
       <c r="B46" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C46" s="3">
         <v>2</v>
@@ -1451,7 +1451,7 @@
         <v>58</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C47" s="3">
         <v>0</v>
@@ -1468,7 +1468,7 @@
         <v>58</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C48" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
Rename AverageGroupsPerIssue --> GroupsPerIssueAverage
</commit_message>
<xml_diff>
--- a/python/pdstools/resources/MetricLimits.xlsx
+++ b/python/pdstools/resources/MetricLimits.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kass1/Documents/Code/pdstools_v4/pega-datascientist-tools/python/pdstools/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanej/Code/pega-datascientist-tools/python/pdstools/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7D033C-1DA4-8543-B0E1-A332D4DD7A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E00337D4-D62E-C148-8F73-AB78BB6E54FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19660" yWindow="-23400" windowWidth="38400" windowHeight="23400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Thresholds" sheetId="1" r:id="rId1"/>
@@ -221,9 +221,6 @@
     <t>ActiveActionCount</t>
   </si>
   <si>
-    <t>AverageGroupsPerIssue</t>
-  </si>
-  <si>
     <t>AverageTreatmentsPerChannelPerAction</t>
   </si>
   <si>
@@ -264,6 +261,9 @@
   </si>
   <si>
     <t>ModelsWithoutResponsesPercentage</t>
+  </si>
+  <si>
+    <t>GroupsPerIssueAverage</t>
   </si>
 </sst>
 </file>
@@ -703,7 +703,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.1640625" bestFit="1" customWidth="1"/>
@@ -827,7 +827,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C6" s="11">
         <v>0.75</v>
@@ -842,7 +842,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C7" s="11">
         <v>0.75</v>
@@ -911,7 +911,7 @@
         <v>19</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C12" s="1">
         <v>-4</v>
@@ -920,7 +920,7 @@
         <v>-2</v>
       </c>
       <c r="G12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H12" s="6"/>
     </row>
@@ -1079,7 +1079,7 @@
         <v>26</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C23" s="10">
         <v>0.5</v>
@@ -1111,7 +1111,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
@@ -1320,7 +1320,7 @@
         <v>58</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C40" s="3">
         <v>1</v>
@@ -1331,6 +1331,7 @@
       <c r="E40" s="3">
         <v>25</v>
       </c>
+      <c r="F40" s="3"/>
       <c r="G40" t="s">
         <v>60</v>
       </c>
@@ -1340,7 +1341,7 @@
         <v>58</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C41" s="3">
         <v>1</v>
@@ -1360,7 +1361,7 @@
         <v>58</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1368,7 +1369,7 @@
         <v>58</v>
       </c>
       <c r="B43" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C43" s="3">
         <v>1</v>
@@ -1385,7 +1386,7 @@
         <v>58</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C44" s="3">
         <v>1</v>
@@ -1405,7 +1406,7 @@
         <v>58</v>
       </c>
       <c r="B45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C45" s="3">
         <v>2</v>
@@ -1428,7 +1429,7 @@
         <v>58</v>
       </c>
       <c r="B46" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C46" s="3">
         <v>2</v>
@@ -1451,7 +1452,7 @@
         <v>58</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C47" s="3">
         <v>0</v>
@@ -1468,7 +1469,7 @@
         <v>58</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C48" s="3">
         <v>0</v>
@@ -1480,9 +1481,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="49" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="8"/>
-    </row>
+    <row r="49" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="8"/>
     </row>
@@ -1502,10 +1501,10 @@
       <c r="A55" s="8"/>
     </row>
     <row r="56" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="9"/>
+      <c r="A56" s="8"/>
     </row>
     <row r="57" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="8"/>
+      <c r="A57" s="9"/>
     </row>
     <row r="58" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="8"/>
@@ -1527,6 +1526,9 @@
     </row>
     <row r="64" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="8"/>
+    </row>
+    <row r="65" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix/metric limit names (#860)
* rename two metric limits to follow conventions

* Auto-export CSV from Excel table

---------

Co-authored-by: github-actions[bot] <github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/python/pdstools/resources/MetricLimits.xlsx
+++ b/python/pdstools/resources/MetricLimits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kass1/Documents/Code/pdstools_v4/pega-datascientist-tools/python/pdstools/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanej/Code/pega-datascientist-tools/python/pdstools/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7D033C-1DA4-8543-B0E1-A332D4DD7A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD10626C-7A66-8949-AD0E-C63600C1C113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="880" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -221,12 +221,6 @@
     <t>ActiveActionCount</t>
   </si>
   <si>
-    <t>AverageGroupsPerIssue</t>
-  </si>
-  <si>
-    <t>AverageTreatmentsPerChannelPerAction</t>
-  </si>
-  <si>
     <t>InactiveActionCount</t>
   </si>
   <si>
@@ -264,6 +258,12 @@
   </si>
   <si>
     <t>ModelsWithoutResponsesPercentage</t>
+  </si>
+  <si>
+    <t>TreatmentsPerChannelPerActionAverage</t>
+  </si>
+  <si>
+    <t>GroupsPerIssueAverage</t>
   </si>
 </sst>
 </file>
@@ -827,7 +827,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C6" s="11">
         <v>0.75</v>
@@ -842,7 +842,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C7" s="11">
         <v>0.75</v>
@@ -911,7 +911,7 @@
         <v>19</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C12" s="1">
         <v>-4</v>
@@ -920,7 +920,7 @@
         <v>-2</v>
       </c>
       <c r="G12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H12" s="6"/>
     </row>
@@ -1079,7 +1079,7 @@
         <v>26</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C23" s="10">
         <v>0.5</v>
@@ -1111,7 +1111,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
@@ -1320,7 +1320,7 @@
         <v>58</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C40" s="3">
         <v>1</v>
@@ -1340,7 +1340,7 @@
         <v>58</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C41" s="3">
         <v>1</v>
@@ -1360,7 +1360,7 @@
         <v>58</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1368,7 +1368,7 @@
         <v>58</v>
       </c>
       <c r="B43" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C43" s="3">
         <v>1</v>
@@ -1385,7 +1385,7 @@
         <v>58</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C44" s="3">
         <v>1</v>
@@ -1405,7 +1405,7 @@
         <v>58</v>
       </c>
       <c r="B45" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C45" s="3">
         <v>2</v>
@@ -1428,7 +1428,7 @@
         <v>58</v>
       </c>
       <c r="B46" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C46" s="3">
         <v>2</v>
@@ -1451,7 +1451,7 @@
         <v>58</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C47" s="3">
         <v>0</v>
@@ -1468,7 +1468,7 @@
         <v>58</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C48" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
update treatment count and average limits to match most recent pega documentation
</commit_message>
<xml_diff>
--- a/python/pdstools/resources/MetricLimits.xlsx
+++ b/python/pdstools/resources/MetricLimits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vanej/Code/pega-datascientist-tools/python/pdstools/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD10626C-7A66-8949-AD0E-C63600C1C113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4860C95-E89C-BA47-ADE4-ECD19A2BD1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="880" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="78">
   <si>
     <t>Category</t>
   </si>
@@ -264,6 +264,9 @@
   </si>
   <si>
     <t>GroupsPerIssueAverage</t>
+  </si>
+  <si>
+    <t>ActiveTreatmentCount</t>
   </si>
 </sst>
 </file>
@@ -274,7 +277,7 @@
     <numFmt numFmtId="164" formatCode="#,##0%"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -320,6 +323,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="6"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -348,7 +358,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -382,6 +392,7 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -400,8 +411,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Thresholds" displayName="Thresholds" ref="A1:G48" totalsRowShown="0">
-  <autoFilter ref="A1:G48" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Thresholds" displayName="Thresholds" ref="A1:G49" totalsRowShown="0">
+  <autoFilter ref="A1:G49" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Category"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="MetricID"/>
@@ -703,7 +714,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.1640625" bestFit="1" customWidth="1"/>
@@ -1339,45 +1350,45 @@
       <c r="A41" t="s">
         <v>58</v>
       </c>
-      <c r="B41" t="s">
-        <v>75</v>
-      </c>
-      <c r="C41" s="3">
-        <v>1</v>
-      </c>
-      <c r="D41" s="3">
-        <v>1</v>
-      </c>
-      <c r="E41" s="3">
-        <v>5</v>
-      </c>
-      <c r="G41" t="s">
-        <v>60</v>
+      <c r="B41" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>58</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>62</v>
+      <c r="B42" t="s">
+        <v>63</v>
+      </c>
+      <c r="C42" s="3">
+        <v>1</v>
+      </c>
+      <c r="D42" s="3">
+        <v>100</v>
+      </c>
+      <c r="E42" s="3">
+        <v>250</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>58</v>
       </c>
-      <c r="B43" t="s">
-        <v>63</v>
+      <c r="B43" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="C43" s="3">
         <v>1</v>
       </c>
       <c r="D43" s="3">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="E43" s="3">
-        <v>250</v>
+        <v>25</v>
+      </c>
+      <c r="G43" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1385,16 +1396,19 @@
         <v>58</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="C44" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" s="3">
-        <v>5</v>
+        <v>2500</v>
       </c>
       <c r="E44" s="3">
-        <v>25</v>
+        <v>5000</v>
+      </c>
+      <c r="F44" s="3">
+        <v>5000</v>
       </c>
       <c r="G44" t="s">
         <v>60</v>
@@ -1404,7 +1418,7 @@
       <c r="A45" t="s">
         <v>58</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="15" t="s">
         <v>65</v>
       </c>
       <c r="C45" s="3">
@@ -1427,7 +1441,7 @@
       <c r="A46" t="s">
         <v>58</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="15" t="s">
         <v>66</v>
       </c>
       <c r="C46" s="3">
@@ -1450,17 +1464,21 @@
       <c r="A47" t="s">
         <v>58</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>67</v>
+      <c r="B47" s="15" t="s">
+        <v>75</v>
       </c>
       <c r="C47" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E47" s="3">
-        <v>50</v>
+        <v>10</v>
+      </c>
+      <c r="F47" s="3"/>
+      <c r="G47" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1468,7 +1486,7 @@
         <v>58</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C48" s="3">
         <v>0</v>
@@ -1480,53 +1498,70 @@
         <v>50</v>
       </c>
     </row>
-    <row r="49" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="8"/>
-    </row>
-    <row r="50" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C49" s="3">
+        <v>0</v>
+      </c>
+      <c r="D49" s="3">
+        <v>1</v>
+      </c>
+      <c r="E49" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="8"/>
     </row>
-    <row r="51" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="8"/>
     </row>
-    <row r="52" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="8"/>
     </row>
-    <row r="53" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="8"/>
     </row>
-    <row r="54" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="8"/>
     </row>
-    <row r="55" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="8"/>
     </row>
-    <row r="56" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="9"/>
-    </row>
-    <row r="57" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="8"/>
-    </row>
-    <row r="58" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="8"/>
+    </row>
+    <row r="57" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="9"/>
+    </row>
+    <row r="58" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="8"/>
     </row>
-    <row r="59" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="8"/>
     </row>
-    <row r="60" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="8"/>
     </row>
-    <row r="61" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="8"/>
     </row>
-    <row r="62" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="8"/>
     </row>
-    <row r="63" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="8"/>
     </row>
-    <row r="64" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="8"/>
+    </row>
+    <row r="65" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A65" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>